<commit_message>
belga és kinálat frissítve
</commit_message>
<xml_diff>
--- a/data/Belga sörök leírás.xlsx
+++ b/data/Belga sörök leírás.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\.weblapkészítés\BagolyPub_webpack\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63B6BDED-885B-407B-BBCD-501F1B1C4A64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E490C29C-9320-4DA7-830A-12524F01201F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="10920" activeTab="2" xr2:uid="{7BEF2045-2184-4FBD-AA18-E05506E1CF75}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" activeTab="2" xr2:uid="{7BEF2045-2184-4FBD-AA18-E05506E1CF75}"/>
   </bookViews>
   <sheets>
     <sheet name="Munka1" sheetId="1" r:id="rId1"/>
@@ -203,18 +203,6 @@
     <t>Sötét vörösesbarna színéhez vastag, drapp hab párosul. Illatából pörkölt aromák bújnak elő némi hideg füstösséggel. Ízében orvosságos-gyógyfüves aromák fedezhetők fel. A karamellmalátának köszönhetően könnyed, aromás, karamelles karakterrel megáldott sör, melynek utóízében enyhe konyakos felhangok jelentkeznek. Sima és szeretetreméltó ital.</t>
   </si>
   <si>
-    <t>La Trappe Blond</t>
-  </si>
-  <si>
-    <t>6,5% Trappista világos ale</t>
-  </si>
-  <si>
-    <t>latrappe-blond.jpg</t>
-  </si>
-  <si>
-    <t>Halvány aranysárga ital hófehér habbal koronázva. A pohárba szagolva kellemes, gyümölcsös illatjegyeket, elsősorban finom szőlőillatot érezhetünk. Ez a lágy gyümölcsösség ízében is folytatódik egy kis mézzel kísérve. A kortyot nagyon kellemes, diszkrét komlókeserűség zárja. Erősen szénsavas, rendkívül könnyed testű, mondjuk úgy: „tapintatos” sör. Azoknak ajánljuk, akik rajonganak a trappista sörök különleges ízvilágáért, de most mégis egy könnyű sörre vágynak.</t>
-  </si>
-  <si>
     <t>Bavaria Apple 0,0%</t>
   </si>
   <si>
@@ -252,6 +240,18 @@
   </si>
   <si>
     <t>Alkoholmentes sör a friss lime és a gyömbér fűszeres ízével, amelyet egyedi receptúra szerint, saját forrásból származó természetes ásványvízzel főznek. Ahol a gyömbér csípőssége felébreszti az ízlelőbimbókat, ott a finom lime teszi teljessé a frissítő élményt. A citrusfélék ízének és a fűszereknek ez az izgalmas keveréke tökéletes szomjoltóként szolgál.</t>
+  </si>
+  <si>
+    <t>5,6% belga IPA Brasserie de Silly</t>
+  </si>
+  <si>
+    <t>Gallica IPA</t>
+  </si>
+  <si>
+    <t>gallica-ipa.jpg</t>
+  </si>
+  <si>
+    <t>Ez a Tomahawk, Cascade, Saaz, Amarillo és Hallertau Blanc komló és két féle enyhén pörkölt maláta felhasználásával készült rézszínű ital a komlófajták találkozásának köszönheti virágos illatát és kiegyensúlyozott ízét. A Nelson Sauvin komlóval történő száraz komlózásnak köszönhetően a Sauvignon Blanc borokra emlékeztető ízjegyekkel is találkozhatunk a korty végén. Egy igazán frissítő ital, melynek színe, illata és íze tökéletes összhangban vannak egymással.</t>
   </si>
 </sst>
 </file>
@@ -323,7 +323,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -340,21 +340,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -1508,13 +1509,13 @@
     <row r="4" spans="2:7" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="2:7" ht="175.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2"/>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
     </row>
     <row r="7" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
@@ -1528,197 +1529,197 @@
       <c r="B9" s="1" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
     </row>
     <row r="14" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="10"/>
+      <c r="C14" s="9"/>
       <c r="D14" s="3"/>
     </row>
     <row r="15" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
     </row>
     <row r="16" spans="2:7" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="2:7" ht="105.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
     </row>
     <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="2:7" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="22" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
     </row>
     <row r="23" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
     </row>
     <row r="24" spans="2:7" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="25" spans="2:7" ht="168.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
     </row>
     <row r="32" spans="2:7" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" spans="2:7" ht="126" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D33" s="8" t="s">
+      <c r="D33" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E33" s="8"/>
-      <c r="F33" s="8"/>
-      <c r="G33" s="8"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
     </row>
     <row r="38" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C38" s="6"/>
-      <c r="D38" s="6"/>
-      <c r="E38" s="6"/>
-      <c r="F38" s="6"/>
-      <c r="G38" s="6"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8"/>
     </row>
     <row r="39" spans="2:7" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" spans="2:7" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D40" s="8" t="s">
+      <c r="D40" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E40" s="8"/>
-      <c r="F40" s="8"/>
-      <c r="G40" s="8"/>
+      <c r="E40" s="6"/>
+      <c r="F40" s="6"/>
+      <c r="G40" s="6"/>
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B45" s="9" t="s">
+      <c r="B45" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C45" s="9"/>
-      <c r="D45" s="9"/>
+      <c r="C45" s="7"/>
+      <c r="D45" s="7"/>
     </row>
     <row r="46" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C46" s="6"/>
-      <c r="D46" s="6"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
     </row>
     <row r="47" spans="2:7" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="48" spans="2:7" ht="190.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D48" s="8" t="s">
+      <c r="D48" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E48" s="8"/>
-      <c r="F48" s="8"/>
-      <c r="G48" s="8"/>
+      <c r="E48" s="6"/>
+      <c r="F48" s="6"/>
+      <c r="G48" s="6"/>
     </row>
     <row r="51" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B51" s="9" t="s">
+      <c r="B51" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C51" s="9"/>
-      <c r="D51" s="9"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="7"/>
     </row>
     <row r="52" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B52" s="6" t="s">
+      <c r="B52" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C52" s="6"/>
-      <c r="D52" s="6"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
     </row>
     <row r="53" spans="2:7" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="54" spans="2:7" ht="159.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D54" s="8" t="s">
+      <c r="D54" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E54" s="8"/>
-      <c r="F54" s="8"/>
-      <c r="G54" s="8"/>
+      <c r="E54" s="6"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="6"/>
     </row>
     <row r="58" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B58" s="9" t="s">
+      <c r="B58" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C58" s="9"/>
-      <c r="D58" s="9"/>
+      <c r="C58" s="7"/>
+      <c r="D58" s="7"/>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B59" s="6" t="s">
+      <c r="B59" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C59" s="6"/>
-      <c r="D59" s="6"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="8"/>
     </row>
     <row r="60" spans="2:7" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="61" spans="2:7" ht="135" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D61" s="8" t="s">
+      <c r="D61" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E61" s="8"/>
-      <c r="F61" s="8"/>
-      <c r="G61" s="8"/>
+      <c r="E61" s="6"/>
+      <c r="F61" s="6"/>
+      <c r="G61" s="6"/>
     </row>
     <row r="64" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="9" t="s">
+      <c r="B64" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C64" s="9"/>
-      <c r="D64" s="9"/>
-      <c r="E64" s="9"/>
+      <c r="C64" s="7"/>
+      <c r="D64" s="7"/>
+      <c r="E64" s="7"/>
     </row>
     <row r="65" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="6" t="s">
+      <c r="B65" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C65" s="6"/>
-      <c r="D65" s="6"/>
-      <c r="E65" s="6"/>
-      <c r="F65" s="6"/>
-      <c r="G65" s="6"/>
+      <c r="C65" s="8"/>
+      <c r="D65" s="8"/>
+      <c r="E65" s="8"/>
+      <c r="F65" s="8"/>
+      <c r="G65" s="8"/>
     </row>
     <row r="66" spans="2:7" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="67" spans="2:7" ht="98.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1730,25 +1731,23 @@
       <c r="G67" s="5"/>
     </row>
     <row r="68" spans="2:7" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D68" s="7" t="s">
+      <c r="D68" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="E68" s="7"/>
-      <c r="F68" s="7"/>
-      <c r="G68" s="7"/>
+      <c r="E68" s="10"/>
+      <c r="F68" s="10"/>
+      <c r="G68" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="D17:G17"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="D25:G25"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B65:G65"/>
+    <mergeCell ref="D67:G67"/>
+    <mergeCell ref="D68:G68"/>
+    <mergeCell ref="D54:G54"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="D61:G61"/>
+    <mergeCell ref="B64:E64"/>
     <mergeCell ref="B52:D52"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B31:D31"/>
@@ -1760,14 +1759,16 @@
     <mergeCell ref="B46:D46"/>
     <mergeCell ref="D48:G48"/>
     <mergeCell ref="B51:D51"/>
-    <mergeCell ref="B65:G65"/>
-    <mergeCell ref="D67:G67"/>
-    <mergeCell ref="D68:G68"/>
-    <mergeCell ref="D54:G54"/>
-    <mergeCell ref="B58:D58"/>
-    <mergeCell ref="B59:D59"/>
-    <mergeCell ref="D61:G61"/>
-    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="D17:G17"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="11" orientation="portrait" r:id="rId1"/>
@@ -1829,44 +1830,44 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" t="s">
         <v>59</v>
-      </c>
-      <c r="B6" t="s">
-        <v>60</v>
-      </c>
-      <c r="C6" t="s">
-        <v>61</v>
-      </c>
-      <c r="D6" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1885,16 +1886,16 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="B8" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1981,9 +1982,15 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C16" s="11"/>
+    </row>
+    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C17" s="11"/>
+    </row>
+    <row r="22" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>